<commit_message>
update resume and make projects printable
</commit_message>
<xml_diff>
--- a/Projects/HUL DCF Valuation/Financial Model and DCF Valuation - HUL.xlsx
+++ b/Projects/HUL DCF Valuation/Financial Model and DCF Valuation - HUL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr showInkAnnotation="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4811e80fe84d3960/Desktop/Finance-Portfolio/Projects/HUL DCF Valuation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\talib\Desktop\Finance-Portfolio\Projects\HUL DCF Valuation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="499" documentId="13_ncr:1_{203CCC4F-8F77-4943-B5E9-2E5C0562AD41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E415522-6EF4-4E05-AD90-BEF98B3B6AD6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{592D0197-1AE6-4592-BF64-DBBDE0C3D740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3782,6 +3782,30 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="94" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="86" fillId="8" borderId="0" xfId="9" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="87" fillId="8" borderId="0" xfId="9" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="83" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3791,18 +3815,6 @@
     <xf numFmtId="0" fontId="81" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="86" fillId="8" borderId="0" xfId="9" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="37" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3815,23 +3827,11 @@
     <xf numFmtId="188" fontId="0" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="82" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="82" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="87" fillId="8" borderId="0" xfId="9" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="173" fontId="94" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -8703,10 +8703,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -9063,21 +9059,21 @@
     </row>
     <row r="3" spans="2:20" ht="15" customHeight="1">
       <c r="B3" s="219"/>
-      <c r="C3" s="491" t="s">
+      <c r="C3" s="499" t="s">
         <v>281</v>
       </c>
-      <c r="D3" s="491"/>
-      <c r="E3" s="491"/>
-      <c r="F3" s="491"/>
-      <c r="G3" s="491"/>
-      <c r="H3" s="491"/>
-      <c r="I3" s="491"/>
-      <c r="J3" s="491"/>
-      <c r="K3" s="491"/>
-      <c r="L3" s="491"/>
-      <c r="M3" s="491"/>
-      <c r="N3" s="491"/>
-      <c r="O3" s="491"/>
+      <c r="D3" s="499"/>
+      <c r="E3" s="499"/>
+      <c r="F3" s="499"/>
+      <c r="G3" s="499"/>
+      <c r="H3" s="499"/>
+      <c r="I3" s="499"/>
+      <c r="J3" s="499"/>
+      <c r="K3" s="499"/>
+      <c r="L3" s="499"/>
+      <c r="M3" s="499"/>
+      <c r="N3" s="499"/>
+      <c r="O3" s="499"/>
       <c r="P3" s="27"/>
       <c r="Q3" s="224"/>
       <c r="R3" s="102"/>
@@ -9085,19 +9081,19 @@
     </row>
     <row r="4" spans="2:20" ht="15" customHeight="1">
       <c r="B4" s="219"/>
-      <c r="C4" s="491"/>
-      <c r="D4" s="491"/>
-      <c r="E4" s="491"/>
-      <c r="F4" s="491"/>
-      <c r="G4" s="491"/>
-      <c r="H4" s="491"/>
-      <c r="I4" s="491"/>
-      <c r="J4" s="491"/>
-      <c r="K4" s="491"/>
-      <c r="L4" s="491"/>
-      <c r="M4" s="491"/>
-      <c r="N4" s="491"/>
-      <c r="O4" s="491"/>
+      <c r="C4" s="499"/>
+      <c r="D4" s="499"/>
+      <c r="E4" s="499"/>
+      <c r="F4" s="499"/>
+      <c r="G4" s="499"/>
+      <c r="H4" s="499"/>
+      <c r="I4" s="499"/>
+      <c r="J4" s="499"/>
+      <c r="K4" s="499"/>
+      <c r="L4" s="499"/>
+      <c r="M4" s="499"/>
+      <c r="N4" s="499"/>
+      <c r="O4" s="499"/>
       <c r="P4" s="27"/>
       <c r="Q4" s="224"/>
       <c r="R4" s="102"/>
@@ -9105,19 +9101,19 @@
     </row>
     <row r="5" spans="2:20" ht="15" customHeight="1">
       <c r="B5" s="219"/>
-      <c r="C5" s="491"/>
-      <c r="D5" s="491"/>
-      <c r="E5" s="491"/>
-      <c r="F5" s="491"/>
-      <c r="G5" s="491"/>
-      <c r="H5" s="491"/>
-      <c r="I5" s="491"/>
-      <c r="J5" s="491"/>
-      <c r="K5" s="491"/>
-      <c r="L5" s="491"/>
-      <c r="M5" s="491"/>
-      <c r="N5" s="491"/>
-      <c r="O5" s="491"/>
+      <c r="C5" s="499"/>
+      <c r="D5" s="499"/>
+      <c r="E5" s="499"/>
+      <c r="F5" s="499"/>
+      <c r="G5" s="499"/>
+      <c r="H5" s="499"/>
+      <c r="I5" s="499"/>
+      <c r="J5" s="499"/>
+      <c r="K5" s="499"/>
+      <c r="L5" s="499"/>
+      <c r="M5" s="499"/>
+      <c r="N5" s="499"/>
+      <c r="O5" s="499"/>
       <c r="P5" s="27"/>
       <c r="Q5" s="224"/>
       <c r="R5" s="223"/>
@@ -9125,19 +9121,19 @@
     </row>
     <row r="6" spans="2:20" ht="15" customHeight="1">
       <c r="B6" s="219"/>
-      <c r="C6" s="491"/>
-      <c r="D6" s="491"/>
-      <c r="E6" s="491"/>
-      <c r="F6" s="491"/>
-      <c r="G6" s="491"/>
-      <c r="H6" s="491"/>
-      <c r="I6" s="491"/>
-      <c r="J6" s="491"/>
-      <c r="K6" s="491"/>
-      <c r="L6" s="491"/>
-      <c r="M6" s="491"/>
-      <c r="N6" s="491"/>
-      <c r="O6" s="491"/>
+      <c r="C6" s="499"/>
+      <c r="D6" s="499"/>
+      <c r="E6" s="499"/>
+      <c r="F6" s="499"/>
+      <c r="G6" s="499"/>
+      <c r="H6" s="499"/>
+      <c r="I6" s="499"/>
+      <c r="J6" s="499"/>
+      <c r="K6" s="499"/>
+      <c r="L6" s="499"/>
+      <c r="M6" s="499"/>
+      <c r="N6" s="499"/>
+      <c r="O6" s="499"/>
       <c r="P6" s="27"/>
       <c r="Q6" s="224"/>
       <c r="R6" s="102"/>
@@ -9145,19 +9141,19 @@
     </row>
     <row r="7" spans="2:20" ht="15" customHeight="1">
       <c r="B7" s="219"/>
-      <c r="C7" s="491"/>
-      <c r="D7" s="491"/>
-      <c r="E7" s="491"/>
-      <c r="F7" s="491"/>
-      <c r="G7" s="491"/>
-      <c r="H7" s="491"/>
-      <c r="I7" s="491"/>
-      <c r="J7" s="491"/>
-      <c r="K7" s="491"/>
-      <c r="L7" s="491"/>
-      <c r="M7" s="491"/>
-      <c r="N7" s="491"/>
-      <c r="O7" s="491"/>
+      <c r="C7" s="499"/>
+      <c r="D7" s="499"/>
+      <c r="E7" s="499"/>
+      <c r="F7" s="499"/>
+      <c r="G7" s="499"/>
+      <c r="H7" s="499"/>
+      <c r="I7" s="499"/>
+      <c r="J7" s="499"/>
+      <c r="K7" s="499"/>
+      <c r="L7" s="499"/>
+      <c r="M7" s="499"/>
+      <c r="N7" s="499"/>
+      <c r="O7" s="499"/>
       <c r="P7" s="27"/>
       <c r="Q7" s="224"/>
       <c r="R7" s="102"/>
@@ -9227,46 +9223,46 @@
     </row>
     <row r="11" spans="2:20" ht="16.5" customHeight="1">
       <c r="B11" s="218"/>
-      <c r="C11" s="492" t="s">
+      <c r="C11" s="500" t="s">
         <v>288</v>
       </c>
-      <c r="D11" s="492"/>
-      <c r="E11" s="492"/>
-      <c r="F11" s="492"/>
-      <c r="G11" s="492"/>
-      <c r="H11" s="492"/>
-      <c r="I11" s="492"/>
+      <c r="D11" s="500"/>
+      <c r="E11" s="500"/>
+      <c r="F11" s="500"/>
+      <c r="G11" s="500"/>
+      <c r="H11" s="500"/>
+      <c r="I11" s="500"/>
       <c r="J11" s="218"/>
       <c r="K11" s="218"/>
       <c r="L11" s="218"/>
       <c r="M11" s="218"/>
-      <c r="N11" s="498" t="s">
+      <c r="N11" s="502" t="s">
         <v>304</v>
       </c>
-      <c r="O11" s="498"/>
-      <c r="P11" s="498"/>
-      <c r="Q11" s="498"/>
-      <c r="R11" s="498"/>
+      <c r="O11" s="502"/>
+      <c r="P11" s="502"/>
+      <c r="Q11" s="502"/>
+      <c r="R11" s="502"/>
       <c r="S11" s="218"/>
     </row>
     <row r="12" spans="2:20" ht="15.75" customHeight="1" thickBot="1">
       <c r="B12" s="218"/>
-      <c r="C12" s="493"/>
-      <c r="D12" s="493"/>
-      <c r="E12" s="493"/>
-      <c r="F12" s="493"/>
-      <c r="G12" s="493"/>
-      <c r="H12" s="493"/>
-      <c r="I12" s="493"/>
+      <c r="C12" s="501"/>
+      <c r="D12" s="501"/>
+      <c r="E12" s="501"/>
+      <c r="F12" s="501"/>
+      <c r="G12" s="501"/>
+      <c r="H12" s="501"/>
+      <c r="I12" s="501"/>
       <c r="J12" s="218"/>
       <c r="K12" s="218"/>
       <c r="L12" s="218"/>
       <c r="M12" s="218"/>
-      <c r="N12" s="499"/>
-      <c r="O12" s="499"/>
-      <c r="P12" s="499"/>
-      <c r="Q12" s="499"/>
-      <c r="R12" s="499"/>
+      <c r="N12" s="503"/>
+      <c r="O12" s="503"/>
+      <c r="P12" s="503"/>
+      <c r="Q12" s="503"/>
+      <c r="R12" s="503"/>
       <c r="S12" s="227"/>
       <c r="T12" s="228"/>
     </row>
@@ -9285,51 +9281,51 @@
       <c r="K13" s="218"/>
       <c r="L13" s="218"/>
       <c r="M13" s="218"/>
-      <c r="N13" s="502" t="s">
+      <c r="N13" s="494" t="s">
         <v>286</v>
       </c>
-      <c r="O13" s="502" t="s">
+      <c r="O13" s="494" t="s">
         <v>300</v>
       </c>
-      <c r="P13" s="502" t="s">
+      <c r="P13" s="494" t="s">
         <v>289</v>
       </c>
-      <c r="Q13" s="502"/>
-      <c r="R13" s="502"/>
+      <c r="Q13" s="494"/>
+      <c r="R13" s="494"/>
       <c r="S13" s="227"/>
       <c r="T13" s="228"/>
     </row>
     <row r="14" spans="2:20" ht="15.75">
       <c r="B14" s="218"/>
-      <c r="C14" s="504" t="s">
+      <c r="C14" s="498" t="s">
         <v>294</v>
       </c>
-      <c r="D14" s="504"/>
-      <c r="E14" s="504"/>
-      <c r="F14" s="504"/>
-      <c r="G14" s="504"/>
-      <c r="H14" s="504"/>
-      <c r="I14" s="504"/>
+      <c r="D14" s="498"/>
+      <c r="E14" s="498"/>
+      <c r="F14" s="498"/>
+      <c r="G14" s="498"/>
+      <c r="H14" s="498"/>
+      <c r="I14" s="498"/>
       <c r="J14" s="218"/>
       <c r="K14" s="218"/>
       <c r="L14" s="218"/>
       <c r="M14" s="218"/>
-      <c r="N14" s="503"/>
-      <c r="O14" s="503"/>
-      <c r="P14" s="503"/>
-      <c r="Q14" s="503"/>
-      <c r="R14" s="503"/>
+      <c r="N14" s="495"/>
+      <c r="O14" s="495"/>
+      <c r="P14" s="495"/>
+      <c r="Q14" s="495"/>
+      <c r="R14" s="495"/>
       <c r="S14" s="227"/>
     </row>
     <row r="15" spans="2:20" ht="15.75">
       <c r="B15" s="218"/>
-      <c r="C15" s="504"/>
-      <c r="D15" s="504"/>
-      <c r="E15" s="504"/>
-      <c r="F15" s="504"/>
-      <c r="G15" s="504"/>
-      <c r="H15" s="504"/>
-      <c r="I15" s="504"/>
+      <c r="C15" s="498"/>
+      <c r="D15" s="498"/>
+      <c r="E15" s="498"/>
+      <c r="F15" s="498"/>
+      <c r="G15" s="498"/>
+      <c r="H15" s="498"/>
+      <c r="I15" s="498"/>
       <c r="J15" s="218"/>
       <c r="K15" s="218"/>
       <c r="L15" s="218"/>
@@ -9349,15 +9345,15 @@
     </row>
     <row r="16" spans="2:20" ht="15.75">
       <c r="B16" s="218"/>
-      <c r="C16" s="494" t="s">
+      <c r="C16" s="492" t="s">
         <v>299</v>
       </c>
-      <c r="D16" s="494"/>
-      <c r="E16" s="494"/>
-      <c r="F16" s="494"/>
-      <c r="G16" s="494"/>
-      <c r="H16" s="494"/>
-      <c r="I16" s="494"/>
+      <c r="D16" s="492"/>
+      <c r="E16" s="492"/>
+      <c r="F16" s="492"/>
+      <c r="G16" s="492"/>
+      <c r="H16" s="492"/>
+      <c r="I16" s="492"/>
       <c r="J16" s="218"/>
       <c r="K16" s="218"/>
       <c r="L16" s="218"/>
@@ -9371,13 +9367,13 @@
     </row>
     <row r="17" spans="2:19" ht="15.75" customHeight="1">
       <c r="B17" s="218"/>
-      <c r="C17" s="494"/>
-      <c r="D17" s="494"/>
-      <c r="E17" s="494"/>
-      <c r="F17" s="494"/>
-      <c r="G17" s="494"/>
-      <c r="H17" s="494"/>
-      <c r="I17" s="494"/>
+      <c r="C17" s="492"/>
+      <c r="D17" s="492"/>
+      <c r="E17" s="492"/>
+      <c r="F17" s="492"/>
+      <c r="G17" s="492"/>
+      <c r="H17" s="492"/>
+      <c r="I17" s="492"/>
       <c r="J17" s="218"/>
       <c r="K17" s="218"/>
       <c r="L17" s="218"/>
@@ -9388,44 +9384,44 @@
       <c r="O17" s="496" t="s">
         <v>300</v>
       </c>
-      <c r="P17" s="500">
+      <c r="P17" s="504">
         <v>46174</v>
       </c>
-      <c r="Q17" s="500"/>
-      <c r="R17" s="500"/>
+      <c r="Q17" s="504"/>
+      <c r="R17" s="504"/>
       <c r="S17" s="227"/>
     </row>
     <row r="18" spans="2:19" ht="15.75" customHeight="1">
       <c r="B18" s="218"/>
-      <c r="C18" s="494" t="s">
+      <c r="C18" s="492" t="s">
         <v>298</v>
       </c>
-      <c r="D18" s="494"/>
-      <c r="E18" s="494"/>
-      <c r="F18" s="494"/>
-      <c r="G18" s="494"/>
-      <c r="H18" s="494"/>
-      <c r="I18" s="494"/>
+      <c r="D18" s="492"/>
+      <c r="E18" s="492"/>
+      <c r="F18" s="492"/>
+      <c r="G18" s="492"/>
+      <c r="H18" s="492"/>
+      <c r="I18" s="492"/>
       <c r="J18" s="218"/>
       <c r="K18" s="218"/>
       <c r="L18" s="218"/>
       <c r="M18" s="218"/>
       <c r="N18" s="497"/>
       <c r="O18" s="497"/>
-      <c r="P18" s="501"/>
-      <c r="Q18" s="501"/>
-      <c r="R18" s="501"/>
+      <c r="P18" s="505"/>
+      <c r="Q18" s="505"/>
+      <c r="R18" s="505"/>
       <c r="S18" s="227"/>
     </row>
     <row r="19" spans="2:19" ht="15.75" customHeight="1">
       <c r="B19" s="218"/>
-      <c r="C19" s="494"/>
-      <c r="D19" s="494"/>
-      <c r="E19" s="494"/>
-      <c r="F19" s="494"/>
-      <c r="G19" s="494"/>
-      <c r="H19" s="494"/>
-      <c r="I19" s="494"/>
+      <c r="C19" s="492"/>
+      <c r="D19" s="492"/>
+      <c r="E19" s="492"/>
+      <c r="F19" s="492"/>
+      <c r="G19" s="492"/>
+      <c r="H19" s="492"/>
+      <c r="I19" s="492"/>
       <c r="J19" s="218"/>
       <c r="K19" s="218"/>
       <c r="L19" s="218"/>
@@ -9445,15 +9441,15 @@
     </row>
     <row r="20" spans="2:19" ht="15.75">
       <c r="B20" s="218"/>
-      <c r="C20" s="494" t="s">
+      <c r="C20" s="492" t="s">
         <v>297</v>
       </c>
-      <c r="D20" s="494"/>
-      <c r="E20" s="494"/>
-      <c r="F20" s="494"/>
-      <c r="G20" s="494"/>
-      <c r="H20" s="494"/>
-      <c r="I20" s="494"/>
+      <c r="D20" s="492"/>
+      <c r="E20" s="492"/>
+      <c r="F20" s="492"/>
+      <c r="G20" s="492"/>
+      <c r="H20" s="492"/>
+      <c r="I20" s="492"/>
       <c r="J20" s="218"/>
       <c r="K20" s="218"/>
       <c r="L20" s="218"/>
@@ -9469,61 +9465,61 @@
     </row>
     <row r="21" spans="2:19" ht="15.75">
       <c r="B21" s="218"/>
-      <c r="C21" s="494"/>
-      <c r="D21" s="494"/>
-      <c r="E21" s="494"/>
-      <c r="F21" s="494"/>
-      <c r="G21" s="494"/>
-      <c r="H21" s="494"/>
-      <c r="I21" s="494"/>
+      <c r="C21" s="492"/>
+      <c r="D21" s="492"/>
+      <c r="E21" s="492"/>
+      <c r="F21" s="492"/>
+      <c r="G21" s="492"/>
+      <c r="H21" s="492"/>
+      <c r="I21" s="492"/>
       <c r="J21" s="218"/>
       <c r="K21" s="218"/>
       <c r="L21" s="218"/>
       <c r="M21" s="218"/>
-      <c r="N21" s="495" t="s">
+      <c r="N21" s="493" t="s">
         <v>287</v>
       </c>
-      <c r="O21" s="495" t="s">
+      <c r="O21" s="493" t="s">
         <v>300</v>
       </c>
-      <c r="P21" s="495" t="s">
+      <c r="P21" s="493" t="s">
         <v>293</v>
       </c>
-      <c r="Q21" s="495"/>
-      <c r="R21" s="495"/>
+      <c r="Q21" s="493"/>
+      <c r="R21" s="493"/>
       <c r="S21" s="227"/>
     </row>
     <row r="22" spans="2:19" ht="15.75">
       <c r="B22" s="218"/>
-      <c r="C22" s="494" t="s">
+      <c r="C22" s="492" t="s">
         <v>296</v>
       </c>
-      <c r="D22" s="494"/>
-      <c r="E22" s="494"/>
-      <c r="F22" s="494"/>
-      <c r="G22" s="494"/>
-      <c r="H22" s="494"/>
-      <c r="I22" s="494"/>
+      <c r="D22" s="492"/>
+      <c r="E22" s="492"/>
+      <c r="F22" s="492"/>
+      <c r="G22" s="492"/>
+      <c r="H22" s="492"/>
+      <c r="I22" s="492"/>
       <c r="J22" s="218"/>
       <c r="K22" s="218"/>
       <c r="L22" s="218"/>
       <c r="M22" s="218"/>
-      <c r="N22" s="495"/>
-      <c r="O22" s="495"/>
-      <c r="P22" s="495"/>
-      <c r="Q22" s="495"/>
-      <c r="R22" s="495"/>
+      <c r="N22" s="493"/>
+      <c r="O22" s="493"/>
+      <c r="P22" s="493"/>
+      <c r="Q22" s="493"/>
+      <c r="R22" s="493"/>
       <c r="S22" s="227"/>
     </row>
     <row r="23" spans="2:19" ht="15.75">
       <c r="B23" s="218"/>
-      <c r="C23" s="494"/>
-      <c r="D23" s="494"/>
-      <c r="E23" s="494"/>
-      <c r="F23" s="494"/>
-      <c r="G23" s="494"/>
-      <c r="H23" s="494"/>
-      <c r="I23" s="494"/>
+      <c r="C23" s="492"/>
+      <c r="D23" s="492"/>
+      <c r="E23" s="492"/>
+      <c r="F23" s="492"/>
+      <c r="G23" s="492"/>
+      <c r="H23" s="492"/>
+      <c r="I23" s="492"/>
       <c r="J23" s="218"/>
       <c r="K23" s="218"/>
       <c r="L23" s="218"/>
@@ -9537,15 +9533,15 @@
     </row>
     <row r="24" spans="2:19" ht="15.75">
       <c r="B24" s="218"/>
-      <c r="C24" s="494" t="s">
+      <c r="C24" s="492" t="s">
         <v>295</v>
       </c>
-      <c r="D24" s="494"/>
-      <c r="E24" s="494"/>
-      <c r="F24" s="494"/>
-      <c r="G24" s="494"/>
-      <c r="H24" s="494"/>
-      <c r="I24" s="494"/>
+      <c r="D24" s="492"/>
+      <c r="E24" s="492"/>
+      <c r="F24" s="492"/>
+      <c r="G24" s="492"/>
+      <c r="H24" s="492"/>
+      <c r="I24" s="492"/>
       <c r="J24" s="218"/>
       <c r="K24" s="218"/>
       <c r="L24" s="218"/>
@@ -9561,13 +9557,13 @@
     </row>
     <row r="25" spans="2:19" ht="15.75">
       <c r="B25" s="218"/>
-      <c r="C25" s="494"/>
-      <c r="D25" s="494"/>
-      <c r="E25" s="494"/>
-      <c r="F25" s="494"/>
-      <c r="G25" s="494"/>
-      <c r="H25" s="494"/>
-      <c r="I25" s="494"/>
+      <c r="C25" s="492"/>
+      <c r="D25" s="492"/>
+      <c r="E25" s="492"/>
+      <c r="F25" s="492"/>
+      <c r="G25" s="492"/>
+      <c r="H25" s="492"/>
+      <c r="I25" s="492"/>
       <c r="J25" s="218"/>
       <c r="K25" s="218"/>
       <c r="L25" s="218"/>
@@ -9583,16 +9579,16 @@
     </row>
     <row r="26" spans="2:19" ht="15.75">
       <c r="B26" s="218"/>
-      <c r="C26" s="494" t="s">
+      <c r="C26" s="492" t="s">
         <v>315</v>
       </c>
-      <c r="D26" s="494"/>
-      <c r="E26" s="494"/>
-      <c r="F26" s="494"/>
-      <c r="G26" s="494"/>
-      <c r="H26" s="494"/>
-      <c r="I26" s="494"/>
-      <c r="J26" s="495"/>
+      <c r="D26" s="492"/>
+      <c r="E26" s="492"/>
+      <c r="F26" s="492"/>
+      <c r="G26" s="492"/>
+      <c r="H26" s="492"/>
+      <c r="I26" s="492"/>
+      <c r="J26" s="493"/>
       <c r="K26" s="218"/>
       <c r="L26" s="218"/>
       <c r="M26" s="218"/>
@@ -9607,14 +9603,14 @@
     </row>
     <row r="27" spans="2:19" ht="15.75">
       <c r="B27" s="218"/>
-      <c r="C27" s="494"/>
-      <c r="D27" s="494"/>
-      <c r="E27" s="494"/>
-      <c r="F27" s="494"/>
-      <c r="G27" s="494"/>
-      <c r="H27" s="494"/>
-      <c r="I27" s="494"/>
-      <c r="J27" s="495"/>
+      <c r="C27" s="492"/>
+      <c r="D27" s="492"/>
+      <c r="E27" s="492"/>
+      <c r="F27" s="492"/>
+      <c r="G27" s="492"/>
+      <c r="H27" s="492"/>
+      <c r="I27" s="492"/>
+      <c r="J27" s="493"/>
       <c r="K27" s="218"/>
       <c r="L27" s="218"/>
       <c r="M27" s="218"/>
@@ -9753,6 +9749,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="C3:O7"/>
+    <mergeCell ref="C11:I12"/>
+    <mergeCell ref="C24:I25"/>
+    <mergeCell ref="O21:O22"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="N11:R12"/>
+    <mergeCell ref="P17:R18"/>
+    <mergeCell ref="P21:R22"/>
     <mergeCell ref="C26:I27"/>
     <mergeCell ref="J26:J27"/>
     <mergeCell ref="P13:R14"/>
@@ -9769,15 +9774,6 @@
     <mergeCell ref="C22:I23"/>
     <mergeCell ref="O15:O16"/>
     <mergeCell ref="O13:O14"/>
-    <mergeCell ref="C3:O7"/>
-    <mergeCell ref="C11:I12"/>
-    <mergeCell ref="C24:I25"/>
-    <mergeCell ref="O21:O22"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="N11:R12"/>
-    <mergeCell ref="P17:R18"/>
-    <mergeCell ref="P21:R22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C14:I15" location="Dashboard!A1" display="Dashboard" xr:uid="{4C84AD9C-54DE-4979-A2DC-ADAF3322820A}"/>
@@ -9788,8 +9784,8 @@
     <hyperlink ref="C24:I25" location="Sensitivity_Analysis!A1" display="Sensitivity_Analysis" xr:uid="{2A70086F-14B6-4479-A857-EA316AADD92E}"/>
     <hyperlink ref="C26:I27" location="Note_and_Sources!A1" display="Notes_and_Sources" xr:uid="{F7E411AE-6BD2-4635-8A7A-3B3BA701C5CA}"/>
   </hyperlinks>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="90" fitToHeight="0" orientation="landscape" verticalDpi="300" r:id="rId1"/>
+  <pageMargins left="0.40157480314960631" right="0.47244094488188981" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="86" fitToHeight="0" orientation="landscape" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10313,8 +10309,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="98" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.40157480314960631" right="0.47244094488188981" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -11467,7 +11463,7 @@
       </c>
       <c r="H58" s="171">
         <f ca="1">TODAY()</f>
-        <v>46199</v>
+        <v>46201</v>
       </c>
     </row>
     <row r="59" spans="2:12">
@@ -11680,8 +11676,8 @@
       <formula>NOT(ISERROR(SEARCH("ERROR",H50)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.40157480314960631" right="0.47244094488188981" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="84" fitToWidth="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -14894,8 +14890,8 @@
       <c r="E110" s="30"/>
     </row>
   </sheetData>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="78" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.40157480314960631" right="0.47244094488188981" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="76" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -19738,8 +19734,8 @@
       <formula>$D$306=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="86" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.40157480314960631" right="0.47244094488188981" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -19756,11 +19752,9 @@
     <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" customWidth="1"/>
-    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.28515625" customWidth="1"/>
+    <col min="9" max="12" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="26.25">
@@ -20609,7 +20603,7 @@
       <c r="F37" s="89"/>
       <c r="G37" s="370">
         <f ca="1">Assumptions!H58</f>
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="H37" s="365">
         <f>Assumptions!H59</f>
@@ -20647,7 +20641,7 @@
       <c r="F38" s="89"/>
       <c r="G38" s="372">
         <f ca="1">G37</f>
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="H38" s="373">
         <f>Assumptions!H60</f>
@@ -20851,7 +20845,7 @@
       <c r="G47" s="56"/>
       <c r="H47" s="482">
         <f ca="1">YEARFRAC(H37,G37)</f>
-        <v>0.51388888888888884</v>
+        <v>0.5083333333333333</v>
       </c>
       <c r="I47" s="482">
         <f>YEARFRAC(I37,H37)</f>
@@ -20893,7 +20887,7 @@
       <c r="G49" s="56"/>
       <c r="H49" s="413">
         <f ca="1">H42*H$47</f>
-        <v>5144.4952628861174</v>
+        <v>5088.8790978819434</v>
       </c>
       <c r="I49" s="413">
         <f>I42*I$47</f>
@@ -20951,7 +20945,7 @@
       </c>
       <c r="H51" s="410">
         <f ca="1">SUM(H49:H50)</f>
-        <v>5144.4952628861174</v>
+        <v>5088.8790978819434</v>
       </c>
       <c r="I51" s="410">
         <f>SUM(I49:I50)</f>
@@ -21009,19 +21003,19 @@
       <c r="G54" s="56"/>
       <c r="H54" s="116">
         <f ca="1">G54+YEARFRAC(H38,G38)</f>
-        <v>1.1111111111111112E-2</v>
+        <v>5.5555555555555558E-3</v>
       </c>
       <c r="I54" s="116">
         <f ca="1">H54+YEARFRAC(I38,H38)</f>
-        <v>1.0111111111111111</v>
+        <v>1.0055555555555555</v>
       </c>
       <c r="J54" s="116">
         <f ca="1">I54+YEARFRAC(J38,I38)</f>
-        <v>2.0111111111111111</v>
+        <v>2.0055555555555555</v>
       </c>
       <c r="K54" s="116">
         <f ca="1">J54+YEARFRAC(K38,J38)</f>
-        <v>3.0111111111111111</v>
+        <v>3.0055555555555555</v>
       </c>
       <c r="L54" s="56"/>
       <c r="M54" s="101"/>
@@ -21051,19 +21045,19 @@
       <c r="G56" s="56"/>
       <c r="H56" s="413">
         <f ca="1">H49/(1+$C$38)^H$54</f>
-        <v>5138.5333911768093</v>
+        <v>5085.9295335626257</v>
       </c>
       <c r="I56" s="413">
         <f ca="1">I49/(1+$C$38)^I$54</f>
-        <v>9866.7473362909786</v>
+        <v>9872.4695166119636</v>
       </c>
       <c r="J56" s="413">
         <f ca="1">J49/(1+$C$38)^J$54</f>
-        <v>9799.2582293788873</v>
+        <v>9804.9412696645286</v>
       </c>
       <c r="K56" s="413">
         <f ca="1">K49/(1+$C$38)^K$54</f>
-        <v>9827.7109971537193</v>
+        <v>9833.4105385072689</v>
       </c>
       <c r="L56" s="56"/>
       <c r="M56" s="101"/>
@@ -21091,7 +21085,7 @@
       </c>
       <c r="K57" s="413">
         <f ca="1">K50/(1+$C$38)^K54</f>
-        <v>118557.54336902931</v>
+        <v>118626.30033811425</v>
       </c>
       <c r="L57" s="56"/>
       <c r="M57" s="101"/>
@@ -21107,19 +21101,19 @@
       <c r="G58" s="56"/>
       <c r="H58" s="410">
         <f ca="1">SUM(H56:H57)</f>
-        <v>5138.5333911768093</v>
+        <v>5085.9295335626257</v>
       </c>
       <c r="I58" s="410">
         <f ca="1">SUM(I56:I57)</f>
-        <v>9866.7473362909786</v>
+        <v>9872.4695166119636</v>
       </c>
       <c r="J58" s="410">
         <f ca="1">SUM(J56:J57)</f>
-        <v>9799.2582293788873</v>
+        <v>9804.9412696645286</v>
       </c>
       <c r="K58" s="410">
         <f ca="1">SUM(K56:K57)</f>
-        <v>128385.25436618303</v>
+        <v>128459.71087662151</v>
       </c>
       <c r="L58" s="56"/>
       <c r="M58" s="101"/>
@@ -21177,7 +21171,7 @@
       <c r="E62" s="383"/>
       <c r="F62" s="424">
         <f ca="1">SUM(H58:K58)</f>
-        <v>153189.79332302971</v>
+        <v>153223.05119646061</v>
       </c>
       <c r="H62" s="382" t="s">
         <v>236</v>
@@ -21185,11 +21179,11 @@
       <c r="I62" s="383"/>
       <c r="J62" s="358">
         <f ca="1">K62/$K$64</f>
-        <v>0.22607413459310394</v>
+        <v>0.2257933815323053</v>
       </c>
       <c r="K62" s="424">
         <f ca="1">SUM(H56:L56)</f>
-        <v>34632.249954000392</v>
+        <v>34596.750858346386</v>
       </c>
       <c r="M62" s="23"/>
     </row>
@@ -21202,7 +21196,7 @@
       <c r="E63" s="385"/>
       <c r="F63" s="485">
         <f ca="1">XNPV(C38,G51:K51,G38:K38)</f>
-        <v>153152.72226023849</v>
+        <v>153184.74112859712</v>
       </c>
       <c r="H63" s="386" t="s">
         <v>238</v>
@@ -21210,11 +21204,11 @@
       <c r="I63" s="169"/>
       <c r="J63" s="359">
         <f ca="1">K63/$K$64</f>
-        <v>0.77392586540689612</v>
+        <v>0.77420661846769467</v>
       </c>
       <c r="K63" s="429">
         <f ca="1">SUM(H57:L57)</f>
-        <v>118557.54336902931</v>
+        <v>118626.30033811425</v>
       </c>
       <c r="M63" s="23"/>
     </row>
@@ -21234,7 +21228,7 @@
       </c>
       <c r="K64" s="483">
         <f ca="1">SUM(K62:K63)</f>
-        <v>153189.79332302971</v>
+        <v>153223.05119646064</v>
       </c>
       <c r="M64" s="23"/>
     </row>
@@ -21275,7 +21269,7 @@
       <c r="E67" s="383"/>
       <c r="F67" s="424">
         <f ca="1">F63</f>
-        <v>153152.72226023849</v>
+        <v>153184.74112859712</v>
       </c>
       <c r="H67" s="382" t="s">
         <v>242</v>
@@ -21284,7 +21278,7 @@
       <c r="J67" s="383"/>
       <c r="K67" s="424">
         <f ca="1">F70</f>
-        <v>164668.20850985398</v>
+        <v>164700.22737821261</v>
       </c>
       <c r="M67" s="23"/>
     </row>
@@ -21326,7 +21320,7 @@
       <c r="J69" s="389"/>
       <c r="K69" s="483">
         <f ca="1">K67/K68</f>
-        <v>700.83767833596073</v>
+        <v>700.97395254193202</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="16.5">
@@ -21338,7 +21332,7 @@
       <c r="E70" s="385"/>
       <c r="F70" s="485">
         <f ca="1">SUM(F67:F69)</f>
-        <v>164668.20850985398</v>
+        <v>164700.22737821261</v>
       </c>
       <c r="G70" s="169"/>
       <c r="H70" s="169"/>
@@ -21458,27 +21452,27 @@
       </c>
       <c r="F77" s="89"/>
       <c r="G77" s="165">
-        <f ca="1">G37</f>
-        <v>46199</v>
+        <f t="shared" ref="G77:L78" ca="1" si="3">G37</f>
+        <v>46201</v>
       </c>
       <c r="H77" s="165">
-        <f>H37</f>
+        <f t="shared" si="3"/>
         <v>46387</v>
       </c>
       <c r="I77" s="399">
-        <f>I37</f>
+        <f t="shared" si="3"/>
         <v>46752</v>
       </c>
       <c r="J77" s="399">
-        <f>J37</f>
+        <f t="shared" si="3"/>
         <v>47118</v>
       </c>
       <c r="K77" s="399">
-        <f>K37</f>
+        <f t="shared" si="3"/>
         <v>47483</v>
       </c>
       <c r="L77" s="400">
-        <f>L37</f>
+        <f t="shared" si="3"/>
         <v>47848</v>
       </c>
     </row>
@@ -21496,27 +21490,27 @@
       </c>
       <c r="F78" s="89"/>
       <c r="G78" s="398">
-        <f ca="1">G38</f>
-        <v>46199</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>46201</v>
       </c>
       <c r="H78" s="398">
-        <f>H38</f>
+        <f t="shared" si="3"/>
         <v>46203</v>
       </c>
       <c r="I78" s="401">
-        <f>I38</f>
+        <f t="shared" si="3"/>
         <v>46568</v>
       </c>
       <c r="J78" s="401">
-        <f>J38</f>
+        <f t="shared" si="3"/>
         <v>46934</v>
       </c>
       <c r="K78" s="401">
-        <f>K38</f>
+        <f t="shared" si="3"/>
         <v>47299</v>
       </c>
       <c r="L78" s="402">
-        <f>L38</f>
+        <f t="shared" si="3"/>
         <v>47664</v>
       </c>
     </row>
@@ -21662,23 +21656,23 @@
       </c>
       <c r="G85" s="56"/>
       <c r="H85" s="410">
-        <f t="shared" ref="H85:L85" si="3">SUM(H83:H84)</f>
+        <f t="shared" ref="H85:L85" si="4">SUM(H83:H84)</f>
         <v>10010.909700751365</v>
       </c>
       <c r="I85" s="410">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10964.79646719206</v>
       </c>
       <c r="J85" s="410">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>12087.67427311414</v>
       </c>
       <c r="K85" s="410">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>13456.276478233227</v>
       </c>
       <c r="L85" s="410">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>162965.98795152252</v>
       </c>
     </row>
@@ -21718,7 +21712,7 @@
       <c r="F88" s="150"/>
       <c r="H88" s="168">
         <f ca="1">YEARFRAC(H77,G77)</f>
-        <v>0.51388888888888884</v>
+        <v>0.5083333333333333</v>
       </c>
       <c r="I88" s="168">
         <f>YEARFRAC(I77,H77)</f>
@@ -21761,7 +21755,7 @@
       <c r="F90" s="150"/>
       <c r="H90" s="413">
         <f ca="1">H83*H88</f>
-        <v>5144.4952628861174</v>
+        <v>5088.8790978819434</v>
       </c>
       <c r="I90" s="413">
         <f>I83*I88</f>
@@ -21822,7 +21816,7 @@
       </c>
       <c r="H92" s="488">
         <f ca="1">SUM(H90:H91)</f>
-        <v>5144.4952628861174</v>
+        <v>5088.8790978819434</v>
       </c>
       <c r="I92" s="488">
         <f>SUM(I90:I91)</f>
@@ -21872,23 +21866,23 @@
       <c r="F95" s="150"/>
       <c r="H95" s="354">
         <f ca="1">G95+YEARFRAC(G78,H78)</f>
-        <v>1.1111111111111112E-2</v>
+        <v>5.5555555555555558E-3</v>
       </c>
       <c r="I95" s="354">
         <f ca="1">H95+YEARFRAC(H78,I78)</f>
-        <v>1.0111111111111111</v>
+        <v>1.0055555555555555</v>
       </c>
       <c r="J95" s="354">
         <f ca="1">I95+YEARFRAC(I78,J78)</f>
-        <v>2.0111111111111111</v>
+        <v>2.0055555555555555</v>
       </c>
       <c r="K95" s="354">
         <f ca="1">J95+YEARFRAC(J78,K78)</f>
-        <v>3.0111111111111111</v>
+        <v>3.0055555555555555</v>
       </c>
       <c r="L95" s="354">
         <f ca="1">K95+YEARFRAC(K78,L78)</f>
-        <v>4.0111111111111111</v>
+        <v>4.0055555555555555</v>
       </c>
     </row>
     <row r="96" spans="2:12" ht="21">
@@ -21901,23 +21895,23 @@
       <c r="F96" s="150"/>
       <c r="H96" s="116">
         <f ca="1">H90/(1+$C$78)^H95</f>
-        <v>5138.5333911768093</v>
+        <v>5085.9295335626257</v>
       </c>
       <c r="I96" s="116">
         <f ca="1">I90/(1+$C$78)^I95</f>
-        <v>9866.7473362909786</v>
+        <v>9872.4695166119636</v>
       </c>
       <c r="J96" s="116">
         <f ca="1">J90/(1+$C$78)^J95</f>
-        <v>9799.2582293788873</v>
+        <v>9804.9412696645286</v>
       </c>
       <c r="K96" s="116">
         <f ca="1">K90/(1+$C$78)^K95</f>
-        <v>9827.7109971537193</v>
+        <v>9833.4105385072689</v>
       </c>
       <c r="L96" s="116">
         <f ca="1">L90/(1+$C$78)^L95</f>
-        <v>9612.7737866780517</v>
+        <v>9618.3486760633168</v>
       </c>
     </row>
     <row r="97" spans="2:12" ht="21">
@@ -21933,20 +21927,20 @@
         <v>0</v>
       </c>
       <c r="I97" s="489">
-        <f t="shared" ref="I97:K97" ca="1" si="4">I91/(1+$C$78)^I95</f>
+        <f t="shared" ref="I97:K97" ca="1" si="5">I91/(1+$C$78)^I95</f>
         <v>0</v>
       </c>
       <c r="J97" s="489">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v>0</v>
       </c>
       <c r="K97" s="489">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v>0</v>
       </c>
       <c r="L97" s="489">
         <f ca="1">L91/(1+$C$78)^L95</f>
-        <v>97613.563181638849</v>
+        <v>97670.173773889896</v>
       </c>
     </row>
     <row r="98" spans="2:12" ht="21">
@@ -21959,23 +21953,23 @@
       <c r="F98" s="150"/>
       <c r="H98" s="410">
         <f ca="1">SUM(H96:H97)</f>
-        <v>5138.5333911768093</v>
+        <v>5085.9295335626257</v>
       </c>
       <c r="I98" s="410">
         <f ca="1">SUM(I96:I97)</f>
-        <v>9866.7473362909786</v>
+        <v>9872.4695166119636</v>
       </c>
       <c r="J98" s="410">
         <f ca="1">SUM(J96:J97)</f>
-        <v>9799.2582293788873</v>
+        <v>9804.9412696645286</v>
       </c>
       <c r="K98" s="410">
         <f ca="1">SUM(K96:K97)</f>
-        <v>9827.7109971537193</v>
+        <v>9833.4105385072689</v>
       </c>
       <c r="L98" s="410">
         <f ca="1">SUM(L96:L97)</f>
-        <v>107226.3369683169</v>
+        <v>107288.52244995322</v>
       </c>
     </row>
     <row r="99" spans="2:12" ht="21">
@@ -22016,7 +22010,7 @@
       <c r="E101" s="392"/>
       <c r="F101" s="424">
         <f ca="1">SUM(H98:L98)</f>
-        <v>141858.58692231728</v>
+        <v>141885.2733082996</v>
       </c>
       <c r="H101" s="382" t="s">
         <v>236</v>
@@ -22024,11 +22018,11 @@
       <c r="I101" s="383"/>
       <c r="J101" s="358">
         <f ca="1">K101/$K$103</f>
-        <v>0.31189528036753472</v>
+        <v>0.31162571353219737</v>
       </c>
       <c r="K101" s="424">
         <f ca="1">SUM(H96:L96)</f>
-        <v>44245.023740678444</v>
+        <v>44215.099534409703</v>
       </c>
     </row>
     <row r="102" spans="2:12" ht="21">
@@ -22040,7 +22034,7 @@
       <c r="E102" s="394"/>
       <c r="F102" s="485">
         <f ca="1">XNPV(C78,G92:L92,G78:L78)</f>
-        <v>141824.57525204727</v>
+        <v>141850.1144290443</v>
       </c>
       <c r="H102" s="386" t="s">
         <v>238</v>
@@ -22048,11 +22042,11 @@
       <c r="I102" s="169"/>
       <c r="J102" s="359">
         <f ca="1">K102/$K$103</f>
-        <v>0.68810471963246533</v>
+        <v>0.68837428646780263</v>
       </c>
       <c r="K102" s="429">
         <f ca="1">SUM(H97:L97)</f>
-        <v>97613.563181638849</v>
+        <v>97670.173773889896</v>
       </c>
     </row>
     <row r="103" spans="2:12" ht="16.5">
@@ -22072,7 +22066,7 @@
       </c>
       <c r="K103" s="483">
         <f ca="1">SUM(K101:K102)</f>
-        <v>141858.58692231728</v>
+        <v>141885.2733082996</v>
       </c>
     </row>
     <row r="104" spans="2:12" ht="16.5">
@@ -22124,7 +22118,7 @@
       <c r="E107" s="395"/>
       <c r="F107" s="424">
         <f ca="1">F102</f>
-        <v>141824.57525204727</v>
+        <v>141850.1144290443</v>
       </c>
       <c r="G107" s="23"/>
       <c r="H107" s="391" t="s">
@@ -22134,7 +22128,7 @@
       <c r="J107" s="395"/>
       <c r="K107" s="424">
         <f ca="1">F110</f>
-        <v>153340.06150166277</v>
+        <v>153365.6006786598</v>
       </c>
     </row>
     <row r="108" spans="2:12" ht="16.5">
@@ -22177,7 +22171,7 @@
       <c r="J109" s="389"/>
       <c r="K109" s="483">
         <f ca="1">K107/K108</f>
-        <v>652.62441166527788</v>
+        <v>652.73310791985659</v>
       </c>
     </row>
     <row r="110" spans="2:12" ht="16.5">
@@ -22189,7 +22183,7 @@
       <c r="E110" s="394"/>
       <c r="F110" s="483">
         <f ca="1">SUM(F107:F109)</f>
-        <v>153340.06150166277</v>
+        <v>153365.6006786598</v>
       </c>
       <c r="G110" s="23"/>
       <c r="H110" s="23"/>
@@ -22209,8 +22203,8 @@
       <formula>H30=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.40157480314960631" right="0.40157480314960631" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="97" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -22385,9 +22379,9 @@
     </row>
     <row r="11" spans="1:22" ht="16.5">
       <c r="A11" s="21"/>
-      <c r="C11" s="507">
+      <c r="C11" s="491">
         <f ca="1">Valuation_DCF!F63</f>
-        <v>153152.72226023849</v>
+        <v>153184.74112859712</v>
       </c>
       <c r="D11" s="199">
         <f>E11-0.005</f>
@@ -22435,7 +22429,7 @@
     </row>
     <row r="12" spans="1:22" ht="16.5" customHeight="1">
       <c r="A12" s="21"/>
-      <c r="B12" s="505" t="s">
+      <c r="B12" s="506" t="s">
         <v>105</v>
       </c>
       <c r="C12" s="199">
@@ -22444,21 +22438,21 @@
       </c>
       <c r="D12" s="437">
         <f t="dataTable" ref="D12:H16" dt2D="1" dtr="1" r1="H56" r2="H57" ca="1"/>
-        <v>176581.6821441527</v>
+        <v>176609.49495312825</v>
       </c>
       <c r="E12" s="438">
-        <v>185971.79462466933</v>
+        <v>186004.0425533719</v>
       </c>
       <c r="F12" s="438">
-        <v>196703.3517452598</v>
+        <v>196740.66838222177</v>
       </c>
       <c r="G12" s="438">
-        <v>209085.9176536334</v>
+        <v>209129.08280012547</v>
       </c>
       <c r="H12" s="439">
-        <v>223532.24454673592</v>
-      </c>
-      <c r="J12" s="506" t="s">
+        <v>223582.23295434643</v>
+      </c>
+      <c r="J12" s="507" t="s">
         <v>105</v>
       </c>
       <c r="K12" s="199">
@@ -22467,218 +22461,218 @@
       </c>
       <c r="L12" s="437">
         <f t="shared" ref="L12:P16" si="0">D12-$H$59+$H$60</f>
-        <v>188097.1683937682</v>
+        <v>188124.98120274374</v>
       </c>
       <c r="M12" s="438">
         <f t="shared" si="0"/>
-        <v>197487.28087428483</v>
+        <v>197519.52880298739</v>
       </c>
       <c r="N12" s="438">
         <f t="shared" si="0"/>
-        <v>208218.8379948753</v>
+        <v>208256.15463183727</v>
       </c>
       <c r="O12" s="438">
         <f t="shared" si="0"/>
-        <v>220601.40390324889</v>
+        <v>220644.56904974097</v>
       </c>
       <c r="P12" s="439">
         <f t="shared" si="0"/>
-        <v>235047.73079635142</v>
+        <v>235097.71920396193</v>
       </c>
       <c r="Q12" s="23"/>
     </row>
     <row r="13" spans="1:22" ht="17.25" customHeight="1">
       <c r="A13" s="184"/>
-      <c r="B13" s="505"/>
+      <c r="B13" s="506"/>
       <c r="C13" s="199">
         <f>C14-0.01</f>
         <v>0.1</v>
       </c>
       <c r="D13" s="440">
-        <v>156972.82530290697</v>
+        <v>156999.2382611252</v>
       </c>
       <c r="E13" s="435">
-        <v>164137.68543494074</v>
+        <v>164167.84120113583</v>
       </c>
       <c r="F13" s="435">
-        <v>172198.15308347868</v>
+        <v>172232.51950864779</v>
       </c>
       <c r="G13" s="435">
-        <v>181333.34975182166</v>
+        <v>181372.48825716131</v>
       </c>
       <c r="H13" s="441">
-        <v>191773.57451564225</v>
-      </c>
-      <c r="J13" s="506"/>
+        <v>191818.16682689107</v>
+      </c>
+      <c r="J13" s="507"/>
       <c r="K13" s="199">
         <f>C13</f>
         <v>0.1</v>
       </c>
       <c r="L13" s="440">
         <f t="shared" si="0"/>
-        <v>168488.31155252247</v>
+        <v>168514.72451074069</v>
       </c>
       <c r="M13" s="435">
         <f t="shared" si="0"/>
-        <v>175653.17168455623</v>
+        <v>175683.32745075133</v>
       </c>
       <c r="N13" s="435">
         <f t="shared" si="0"/>
-        <v>183713.63933309418</v>
+        <v>183748.00575826329</v>
       </c>
       <c r="O13" s="435">
         <f t="shared" si="0"/>
-        <v>192848.83600143716</v>
+        <v>192887.97450677681</v>
       </c>
       <c r="P13" s="441">
         <f t="shared" si="0"/>
-        <v>203289.06076525775</v>
+        <v>203333.65307650657</v>
       </c>
       <c r="Q13" s="23"/>
     </row>
     <row r="14" spans="1:22" ht="21">
       <c r="A14" s="184"/>
-      <c r="B14" s="505"/>
+      <c r="B14" s="506"/>
       <c r="C14" s="297">
         <f>Assumptions!H43</f>
         <v>0.11</v>
       </c>
       <c r="D14" s="440">
-        <v>141300.1689422623</v>
+        <v>141325.40815925412</v>
       </c>
       <c r="E14" s="435">
-        <v>146914.53630340891</v>
+        <v>146942.98693420607</v>
       </c>
       <c r="F14" s="472">
-        <v>153152.72226023849</v>
+        <v>153184.74112859712</v>
       </c>
       <c r="G14" s="435">
-        <v>160124.81244728333</v>
+        <v>160160.81934585772</v>
       </c>
       <c r="H14" s="441">
-        <v>167968.41390770872</v>
-      </c>
-      <c r="J14" s="506"/>
+        <v>168008.90734027585</v>
+      </c>
+      <c r="J14" s="507"/>
       <c r="K14" s="199">
         <f>C14</f>
         <v>0.11</v>
       </c>
       <c r="L14" s="440">
         <f t="shared" si="0"/>
-        <v>152815.6551918778</v>
+        <v>152840.89440886962</v>
       </c>
       <c r="M14" s="435">
         <f t="shared" si="0"/>
-        <v>158430.02255302441</v>
+        <v>158458.47318382157</v>
       </c>
       <c r="N14" s="472">
         <f t="shared" si="0"/>
-        <v>164668.20850985398</v>
+        <v>164700.22737821261</v>
       </c>
       <c r="O14" s="435">
         <f t="shared" si="0"/>
-        <v>171640.29869689883</v>
+        <v>171676.30559547321</v>
       </c>
       <c r="P14" s="441">
         <f t="shared" si="0"/>
-        <v>179483.90015732421</v>
+        <v>179524.39358989135</v>
       </c>
       <c r="Q14" s="14"/>
     </row>
     <row r="15" spans="1:22" ht="16.5">
       <c r="A15" s="187"/>
-      <c r="B15" s="505"/>
+      <c r="B15" s="506"/>
       <c r="C15" s="199">
         <f>C14+0.01</f>
         <v>0.12</v>
       </c>
       <c r="D15" s="440">
-        <v>128489.68764368931</v>
+        <v>128513.92019362724</v>
       </c>
       <c r="E15" s="435">
-        <v>132984.42126748073</v>
+        <v>133011.44581984606</v>
       </c>
       <c r="F15" s="435">
-        <v>137928.62825365129</v>
+        <v>137958.72400868672</v>
       </c>
       <c r="G15" s="435">
-        <v>143393.27808047135</v>
+        <v>143426.76832266856</v>
       </c>
       <c r="H15" s="441">
-        <v>149465.1112213826</v>
-      </c>
-      <c r="J15" s="506"/>
+        <v>149502.3731159817</v>
+      </c>
+      <c r="J15" s="507"/>
       <c r="K15" s="199">
         <f>C15</f>
         <v>0.12</v>
       </c>
       <c r="L15" s="440">
         <f t="shared" si="0"/>
-        <v>140005.17389330477</v>
+        <v>140029.40644324271</v>
       </c>
       <c r="M15" s="435">
         <f t="shared" si="0"/>
-        <v>144499.90751709623</v>
+        <v>144526.93206946156</v>
       </c>
       <c r="N15" s="435">
         <f t="shared" si="0"/>
-        <v>149444.11450326678</v>
+        <v>149474.21025830222</v>
       </c>
       <c r="O15" s="435">
         <f t="shared" si="0"/>
-        <v>154908.76433008685</v>
+        <v>154942.25457228406</v>
       </c>
       <c r="P15" s="441">
         <f t="shared" si="0"/>
-        <v>160980.59747099809</v>
+        <v>161017.85936559719</v>
       </c>
       <c r="Q15" s="14"/>
     </row>
     <row r="16" spans="1:22" ht="15.75">
-      <c r="B16" s="505"/>
+      <c r="B16" s="506"/>
       <c r="C16" s="199">
         <f>C15+0.01</f>
         <v>0.13</v>
       </c>
       <c r="D16" s="442">
-        <v>117825.3874735244</v>
+        <v>117848.74094062693</v>
       </c>
       <c r="E16" s="443">
-        <v>121487.84596817169</v>
+        <v>121513.65295265488</v>
       </c>
       <c r="F16" s="443">
-        <v>125483.25523505962</v>
+        <v>125511.73878395811</v>
       </c>
       <c r="G16" s="443">
-        <v>129859.17967022257</v>
+        <v>129890.59469443306</v>
       </c>
       <c r="H16" s="444">
-        <v>134672.69654890185</v>
-      </c>
-      <c r="J16" s="506"/>
+        <v>134707.33619595552</v>
+      </c>
+      <c r="J16" s="507"/>
       <c r="K16" s="199">
         <f>C16</f>
         <v>0.13</v>
       </c>
       <c r="L16" s="442">
         <f t="shared" si="0"/>
-        <v>129340.87372313988</v>
+        <v>129364.22719024241</v>
       </c>
       <c r="M16" s="443">
         <f t="shared" si="0"/>
-        <v>133003.33221778716</v>
+        <v>133029.13920227037</v>
       </c>
       <c r="N16" s="443">
         <f t="shared" si="0"/>
-        <v>136998.74148467509</v>
+        <v>137027.22503357357</v>
       </c>
       <c r="O16" s="443">
         <f t="shared" si="0"/>
-        <v>141374.66591983804</v>
+        <v>141406.08094404853</v>
       </c>
       <c r="P16" s="444">
         <f t="shared" si="0"/>
-        <v>146188.18279851734</v>
+        <v>146222.82244557102</v>
       </c>
       <c r="Q16" s="186"/>
     </row>
@@ -22800,7 +22794,7 @@
       </c>
     </row>
     <row r="23" spans="2:17" ht="20.25" customHeight="1">
-      <c r="B23" s="505" t="s">
+      <c r="B23" s="506" t="s">
         <v>105</v>
       </c>
       <c r="C23" s="199">
@@ -22809,26 +22803,26 @@
       </c>
       <c r="D23" s="437">
         <f t="shared" ref="D23:H27" si="1">L12/$H$61</f>
-        <v>800.55272351352573</v>
+        <v>800.67109648088126</v>
       </c>
       <c r="E23" s="438">
         <f t="shared" si="1"/>
-        <v>840.51760009603254</v>
+        <v>840.65484919643609</v>
       </c>
       <c r="F23" s="438">
         <f t="shared" si="1"/>
-        <v>886.19174476175465</v>
+        <v>886.35056658564167</v>
       </c>
       <c r="G23" s="438">
         <f t="shared" si="1"/>
-        <v>938.89268091451095</v>
+        <v>939.0763943424173</v>
       </c>
       <c r="H23" s="439">
         <f t="shared" si="1"/>
-        <v>1000.3771064260599</v>
+        <v>1000.5898600586553</v>
       </c>
       <c r="I23" s="169"/>
-      <c r="J23" s="506" t="s">
+      <c r="J23" s="507" t="s">
         <v>105</v>
       </c>
       <c r="K23" s="214">
@@ -22837,235 +22831,235 @@
       </c>
       <c r="L23" s="445">
         <f t="shared" ref="L23:P27" si="2">$H$62/D23</f>
-        <v>2.7481013247253414</v>
+        <v>2.7476950394106456</v>
       </c>
       <c r="M23" s="446">
         <f t="shared" si="2"/>
-        <v>2.6174347803646718</v>
+        <v>2.6170074461628725</v>
       </c>
       <c r="N23" s="446">
         <f t="shared" si="2"/>
-        <v>2.4825327171056553</v>
+        <v>2.4820878814064931</v>
       </c>
       <c r="O23" s="446">
         <f t="shared" si="2"/>
-        <v>2.3431858025106034</v>
+        <v>2.3427274002990321</v>
       </c>
       <c r="P23" s="447">
         <f t="shared" si="2"/>
-        <v>2.1991706786050957</v>
+        <v>2.1987030728764676</v>
       </c>
     </row>
     <row r="24" spans="2:17" ht="16.5">
-      <c r="B24" s="505"/>
+      <c r="B24" s="506"/>
       <c r="C24" s="199">
         <f>K13</f>
         <v>0.1</v>
       </c>
       <c r="D24" s="440">
         <f t="shared" si="1"/>
-        <v>717.09626383740988</v>
+        <v>717.20867895677725</v>
       </c>
       <c r="E24" s="435">
         <f t="shared" si="1"/>
-        <v>747.59033422280515</v>
+        <v>747.7186789552818</v>
       </c>
       <c r="F24" s="435">
         <f t="shared" si="1"/>
-        <v>781.89616340637463</v>
+        <v>782.04242895359937</v>
       </c>
       <c r="G24" s="435">
         <f t="shared" si="1"/>
-        <v>820.77610314775325</v>
+        <v>820.94267895169253</v>
       </c>
       <c r="H24" s="441">
         <f t="shared" si="1"/>
-        <v>865.21031999504328</v>
+        <v>865.40010752094202</v>
       </c>
       <c r="I24" s="169"/>
-      <c r="J24" s="506"/>
+      <c r="J24" s="507"/>
       <c r="K24" s="214">
         <f>C24</f>
         <v>0.1</v>
       </c>
       <c r="L24" s="448">
         <f t="shared" si="2"/>
-        <v>3.0679284092586134</v>
+        <v>3.0674475428825416</v>
       </c>
       <c r="M24" s="449">
         <f t="shared" si="2"/>
-        <v>2.9427881812933281</v>
+        <v>2.9422830563412656</v>
       </c>
       <c r="N24" s="449">
         <f t="shared" si="2"/>
-        <v>2.8136728416924011</v>
+        <v>2.8131465999148899</v>
       </c>
       <c r="O24" s="449">
         <f t="shared" si="2"/>
-        <v>2.6803899279752343</v>
+        <v>2.6798460555240013</v>
       </c>
       <c r="P24" s="450">
         <f t="shared" si="2"/>
-        <v>2.5427343492766057</v>
+        <v>2.5421767121132022</v>
       </c>
     </row>
     <row r="25" spans="2:17" ht="16.5">
-      <c r="B25" s="505"/>
+      <c r="B25" s="506"/>
       <c r="C25" s="199">
         <f>K14</f>
         <v>0.11</v>
       </c>
       <c r="D25" s="440">
         <f t="shared" si="1"/>
-        <v>650.39250725591864</v>
+        <v>650.49992686289465</v>
       </c>
       <c r="E25" s="435">
         <f t="shared" si="1"/>
-        <v>674.28758829383332</v>
+        <v>674.40867586875447</v>
       </c>
       <c r="F25" s="472">
         <f t="shared" si="1"/>
-        <v>700.83767833596073</v>
+        <v>700.97395254193202</v>
       </c>
       <c r="G25" s="435">
         <f t="shared" si="1"/>
-        <v>730.51130838304437</v>
+        <v>730.66455588254234</v>
       </c>
       <c r="H25" s="441">
         <f t="shared" si="1"/>
-        <v>763.89414218601326</v>
+        <v>764.06648464072885</v>
       </c>
       <c r="I25" s="169"/>
-      <c r="J25" s="506"/>
+      <c r="J25" s="507"/>
       <c r="K25" s="214">
         <f>C25</f>
         <v>0.11</v>
       </c>
       <c r="L25" s="448">
         <f t="shared" si="2"/>
-        <v>3.3825727932845582</v>
+        <v>3.382014215758232</v>
       </c>
       <c r="M25" s="449">
         <f t="shared" si="2"/>
-        <v>3.2627027965422215</v>
+        <v>3.2621169903634786</v>
       </c>
       <c r="N25" s="473">
         <f t="shared" si="2"/>
-        <v>3.1391006334356719</v>
+        <v>3.1384903704655085</v>
       </c>
       <c r="O25" s="449">
         <f t="shared" si="2"/>
-        <v>3.0115892454418072</v>
+        <v>3.0109576033049836</v>
       </c>
       <c r="P25" s="450">
         <f t="shared" si="2"/>
-        <v>2.8799801942509013</v>
+        <v>2.8793305873564923</v>
       </c>
     </row>
     <row r="26" spans="2:17" ht="16.5">
-      <c r="B26" s="505"/>
+      <c r="B26" s="506"/>
       <c r="C26" s="199">
         <f>K15</f>
         <v>0.12</v>
       </c>
       <c r="D26" s="440">
         <f t="shared" si="1"/>
-        <v>595.87033778007287</v>
+        <v>595.97347295226155</v>
       </c>
       <c r="E26" s="435">
         <f t="shared" si="1"/>
-        <v>615.00019111450138</v>
+        <v>615.11520921489353</v>
       </c>
       <c r="F26" s="435">
         <f t="shared" si="1"/>
-        <v>636.0430297823724</v>
+        <v>636.17111910378833</v>
       </c>
       <c r="G26" s="435">
         <f t="shared" si="1"/>
-        <v>659.30090409949298</v>
+        <v>659.44344055993542</v>
       </c>
       <c r="H26" s="441">
         <f t="shared" si="1"/>
-        <v>685.14298667407161</v>
+        <v>685.30157551120988</v>
       </c>
       <c r="I26" s="169"/>
-      <c r="J26" s="506"/>
+      <c r="J26" s="507"/>
       <c r="K26" s="214">
         <f>C26</f>
         <v>0.12</v>
       </c>
       <c r="L26" s="448">
         <f t="shared" si="2"/>
-        <v>3.6920783944308169</v>
+        <v>3.6914394681056946</v>
       </c>
       <c r="M26" s="449">
         <f t="shared" si="2"/>
-        <v>3.5772346607131409</v>
+        <v>3.5765657669365467</v>
       </c>
       <c r="N26" s="449">
         <f t="shared" si="2"/>
-        <v>3.4588854794191346</v>
+        <v>3.4581890531265698</v>
       </c>
       <c r="O26" s="449">
         <f t="shared" si="2"/>
-        <v>3.3368678646131587</v>
+        <v>3.3361466119550349</v>
       </c>
       <c r="P26" s="450">
         <f t="shared" si="2"/>
-        <v>3.2110085672475237</v>
+        <v>3.2102654927633583</v>
       </c>
     </row>
     <row r="27" spans="2:17" ht="16.5">
-      <c r="B27" s="505"/>
+      <c r="B27" s="506"/>
       <c r="C27" s="199">
         <f>K16</f>
         <v>0.13</v>
       </c>
       <c r="D27" s="442">
         <f t="shared" si="1"/>
-        <v>550.4824426910892</v>
+        <v>550.58183643450411</v>
       </c>
       <c r="E27" s="443">
         <f t="shared" si="1"/>
-        <v>566.07008363051682</v>
+        <v>566.17991968966714</v>
       </c>
       <c r="F27" s="443">
         <f t="shared" si="1"/>
-        <v>583.07478283716523</v>
+        <v>583.19601051348127</v>
       </c>
       <c r="G27" s="443">
         <f t="shared" si="1"/>
-        <v>601.6989772063514</v>
+        <v>601.832681415754</v>
       </c>
       <c r="H27" s="444">
         <f t="shared" si="1"/>
-        <v>622.18559101245648</v>
+        <v>622.33301940825413</v>
       </c>
       <c r="I27" s="169"/>
-      <c r="J27" s="506"/>
+      <c r="J27" s="507"/>
       <c r="K27" s="214">
         <f>C27</f>
         <v>0.13</v>
       </c>
       <c r="L27" s="451">
         <f t="shared" si="2"/>
-        <v>3.9964944008842083</v>
+        <v>3.9957729340417618</v>
       </c>
       <c r="M27" s="452">
         <f t="shared" si="2"/>
-        <v>3.8864445651149726</v>
+        <v>3.8856906144002026</v>
       </c>
       <c r="N27" s="452">
         <f t="shared" si="2"/>
-        <v>3.7731009207688406</v>
+        <v>3.7723166145512312</v>
       </c>
       <c r="O27" s="452">
         <f t="shared" si="2"/>
-        <v>3.6563133449460969</v>
+        <v>3.6555010519281037</v>
       </c>
       <c r="P27" s="453">
         <f t="shared" si="2"/>
-        <v>3.5359224510809266</v>
+        <v>3.5350848041003382</v>
       </c>
     </row>
     <row r="28" spans="2:17" ht="16.5">
@@ -23183,9 +23177,9 @@
       <c r="P34" s="179"/>
     </row>
     <row r="35" spans="1:16" ht="16.5">
-      <c r="C35" s="507">
+      <c r="C35" s="491">
         <f ca="1">Valuation_DCF!F102</f>
-        <v>141824.57525204727</v>
+        <v>141850.1144290443</v>
       </c>
       <c r="D35" s="206">
         <f>E35-0.5</f>
@@ -23231,7 +23225,7 @@
       </c>
     </row>
     <row r="36" spans="1:16" ht="16.5" customHeight="1">
-      <c r="B36" s="505" t="s">
+      <c r="B36" s="506" t="s">
         <v>105</v>
       </c>
       <c r="C36" s="199">
@@ -23240,21 +23234,21 @@
       </c>
       <c r="D36" s="437">
         <f t="dataTable" ref="D36:H40" dt2D="1" dtr="1" r1="H58" r2="H57" ca="1"/>
-        <v>136868.27466823498</v>
+        <v>136877.3301175636</v>
       </c>
       <c r="E36" s="438">
-        <v>144434.98643666593</v>
+        <v>144447.61578063128</v>
       </c>
       <c r="F36" s="438">
-        <v>152001.69820509688</v>
+        <v>152017.901443699</v>
       </c>
       <c r="G36" s="438">
-        <v>159568.40997352783</v>
+        <v>159588.18710676668</v>
       </c>
       <c r="H36" s="439">
-        <v>167135.12174195878</v>
-      </c>
-      <c r="J36" s="506" t="s">
+        <v>167158.47276983439</v>
+      </c>
+      <c r="J36" s="507" t="s">
         <v>105</v>
       </c>
       <c r="K36" s="199">
@@ -23263,211 +23257,211 @@
       </c>
       <c r="L36" s="454">
         <f t="shared" ref="L36:P40" si="3">D36-$H$59+$H$60</f>
-        <v>148383.76091785048</v>
+        <v>148392.8163671791</v>
       </c>
       <c r="M36" s="455">
         <f t="shared" si="3"/>
-        <v>155950.47268628143</v>
+        <v>155963.10203024678</v>
       </c>
       <c r="N36" s="455">
         <f t="shared" si="3"/>
-        <v>163517.18445471238</v>
+        <v>163533.38769331449</v>
       </c>
       <c r="O36" s="455">
         <f t="shared" si="3"/>
-        <v>171083.89622314333</v>
+        <v>171103.67335638218</v>
       </c>
       <c r="P36" s="456">
         <f t="shared" si="3"/>
-        <v>178650.60799157427</v>
+        <v>178673.95901944989</v>
       </c>
     </row>
     <row r="37" spans="1:16">
-      <c r="B37" s="505"/>
+      <c r="B37" s="506"/>
       <c r="C37" s="199">
         <f>C38-0.01</f>
         <v>0.1</v>
       </c>
       <c r="D37" s="440">
-        <v>132269.59367331112</v>
+        <v>132283.10205967524</v>
       </c>
       <c r="E37" s="435">
-        <v>139530.73713349778</v>
+        <v>139548.03862470461</v>
       </c>
       <c r="F37" s="435">
-        <v>146791.88059368441</v>
+        <v>146812.97518973396</v>
       </c>
       <c r="G37" s="435">
-        <v>154053.02405387105</v>
+        <v>154077.91175476328</v>
       </c>
       <c r="H37" s="441">
-        <v>161314.16751405771</v>
-      </c>
-      <c r="J37" s="506"/>
+        <v>161342.84831979265</v>
+      </c>
+      <c r="J37" s="507"/>
       <c r="K37" s="199">
         <f>C37</f>
         <v>0.1</v>
       </c>
       <c r="L37" s="457">
         <f t="shared" si="3"/>
-        <v>143785.07992292658</v>
+        <v>143798.5883092907</v>
       </c>
       <c r="M37" s="458">
         <f t="shared" si="3"/>
-        <v>151046.22338311328</v>
+        <v>151063.52487432011</v>
       </c>
       <c r="N37" s="458">
         <f t="shared" si="3"/>
-        <v>158307.36684329991</v>
+        <v>158328.46143934946</v>
       </c>
       <c r="O37" s="458">
         <f t="shared" si="3"/>
-        <v>165568.51030348655</v>
+        <v>165593.39800437877</v>
       </c>
       <c r="P37" s="459">
         <f t="shared" si="3"/>
-        <v>172829.65376367321</v>
+        <v>172858.33456940815</v>
       </c>
     </row>
     <row r="38" spans="1:16">
-      <c r="B38" s="505"/>
+      <c r="B38" s="506"/>
       <c r="C38" s="297">
         <f>Assumptions!H43</f>
         <v>0.11</v>
       </c>
       <c r="D38" s="440">
-        <v>127883.54556552669</v>
+        <v>127901.11048428307</v>
       </c>
       <c r="E38" s="435">
-        <v>134854.06040878699</v>
+        <v>134875.61245666369</v>
       </c>
       <c r="F38" s="472">
-        <v>141824.57525204727</v>
+        <v>141850.1144290443</v>
       </c>
       <c r="G38" s="435">
-        <v>148795.09009530756</v>
+        <v>148824.61640142492</v>
       </c>
       <c r="H38" s="441">
-        <v>155765.60493856788</v>
-      </c>
-      <c r="J38" s="506"/>
+        <v>155799.11837380557</v>
+      </c>
+      <c r="J38" s="507"/>
       <c r="K38" s="209">
         <f>C38</f>
         <v>0.11</v>
       </c>
       <c r="L38" s="457">
         <f t="shared" si="3"/>
-        <v>139399.03181514217</v>
+        <v>139416.59673389854</v>
       </c>
       <c r="M38" s="458">
         <f t="shared" si="3"/>
-        <v>146369.54665840248</v>
+        <v>146391.09870627918</v>
       </c>
       <c r="N38" s="474">
         <f t="shared" si="3"/>
-        <v>153340.06150166277</v>
+        <v>153365.6006786598</v>
       </c>
       <c r="O38" s="458">
         <f t="shared" si="3"/>
-        <v>160310.57634492306</v>
+        <v>160340.10265104042</v>
       </c>
       <c r="P38" s="459">
         <f t="shared" si="3"/>
-        <v>167281.09118818337</v>
+        <v>167314.60462342107</v>
       </c>
     </row>
     <row r="39" spans="1:16">
-      <c r="B39" s="505"/>
+      <c r="B39" s="506"/>
       <c r="C39" s="199">
         <f>C38+0.01</f>
         <v>0.12</v>
       </c>
       <c r="D39" s="440">
-        <v>123698.31711999365</v>
+        <v>123719.57340498411</v>
       </c>
       <c r="E39" s="435">
-        <v>130392.28774306487</v>
+        <v>130417.7021348071</v>
       </c>
       <c r="F39" s="435">
-        <v>137086.25836613605</v>
+        <v>137115.83086463006</v>
       </c>
       <c r="G39" s="435">
-        <v>143780.22898920727</v>
+        <v>143813.95959445304</v>
       </c>
       <c r="H39" s="441">
-        <v>150474.19961227849</v>
-      </c>
-      <c r="J39" s="506"/>
+        <v>150512.08832427603</v>
+      </c>
+      <c r="J39" s="507"/>
       <c r="K39" s="199">
         <f>C39</f>
         <v>0.12</v>
       </c>
       <c r="L39" s="457">
         <f t="shared" si="3"/>
-        <v>135213.80336960912</v>
+        <v>135235.05965459958</v>
       </c>
       <c r="M39" s="458">
         <f t="shared" si="3"/>
-        <v>141907.77399268033</v>
+        <v>141933.18838442257</v>
       </c>
       <c r="N39" s="458">
         <f t="shared" si="3"/>
-        <v>148601.74461575155</v>
+        <v>148631.31711424555</v>
       </c>
       <c r="O39" s="458">
         <f t="shared" si="3"/>
-        <v>155295.71523882277</v>
+        <v>155329.44584406854</v>
       </c>
       <c r="P39" s="459">
         <f t="shared" si="3"/>
-        <v>161989.68586189399</v>
+        <v>162027.57457389153</v>
       </c>
     </row>
     <row r="40" spans="1:16">
-      <c r="B40" s="505"/>
+      <c r="B40" s="506"/>
       <c r="C40" s="199">
         <f>C39+0.01</f>
         <v>0.13</v>
       </c>
       <c r="D40" s="442">
-        <v>119702.85387533896</v>
+        <v>119727.46507586158</v>
       </c>
       <c r="E40" s="443">
-        <v>126133.56536978636</v>
+        <v>126162.48456791355</v>
       </c>
       <c r="F40" s="443">
-        <v>132564.27686423372</v>
+        <v>132597.50405996549</v>
       </c>
       <c r="G40" s="443">
-        <v>138994.98835868109</v>
+        <v>139032.52355201746</v>
       </c>
       <c r="H40" s="444">
-        <v>145425.69985312849</v>
-      </c>
-      <c r="J40" s="506"/>
+        <v>145467.54304406943</v>
+      </c>
+      <c r="J40" s="507"/>
       <c r="K40" s="199">
         <f>C40</f>
         <v>0.13</v>
       </c>
       <c r="L40" s="460">
         <f t="shared" si="3"/>
-        <v>131218.34012495444</v>
+        <v>131242.95132547704</v>
       </c>
       <c r="M40" s="461">
         <f t="shared" si="3"/>
-        <v>137649.05161940184</v>
+        <v>137677.97081752901</v>
       </c>
       <c r="N40" s="461">
         <f t="shared" si="3"/>
-        <v>144079.76311384921</v>
+        <v>144112.99030958099</v>
       </c>
       <c r="O40" s="461">
         <f t="shared" si="3"/>
-        <v>150510.47460829659</v>
+        <v>150548.00980163296</v>
       </c>
       <c r="P40" s="462">
         <f t="shared" si="3"/>
-        <v>156941.18610274399</v>
+        <v>156983.02929368493</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="16.5">
@@ -23580,7 +23574,7 @@
       </c>
     </row>
     <row r="47" spans="1:16" ht="16.5" customHeight="1">
-      <c r="B47" s="505" t="s">
+      <c r="B47" s="506" t="s">
         <v>105</v>
       </c>
       <c r="C47" s="199">
@@ -23589,25 +23583,25 @@
       </c>
       <c r="D47" s="454">
         <f t="shared" ref="D47:H51" si="4">L36/$H$61</f>
-        <v>631.5301019273644</v>
+        <v>631.5686424576902</v>
       </c>
       <c r="E47" s="455">
         <f t="shared" si="4"/>
-        <v>663.73447675122247</v>
+        <v>663.7882279894468</v>
       </c>
       <c r="F47" s="455">
         <f t="shared" si="4"/>
-        <v>695.93885157508043</v>
+        <v>696.00781352120339</v>
       </c>
       <c r="G47" s="455">
         <f t="shared" si="4"/>
-        <v>728.1432263989384</v>
+        <v>728.22739905295998</v>
       </c>
       <c r="H47" s="456">
         <f t="shared" si="4"/>
-        <v>760.34760122279636</v>
-      </c>
-      <c r="J47" s="506" t="s">
+        <v>760.44698458471669</v>
+      </c>
+      <c r="J47" s="507" t="s">
         <v>105</v>
       </c>
       <c r="K47" s="199">
@@ -23616,231 +23610,231 @@
       </c>
       <c r="L47" s="463">
         <f t="shared" ref="L47:P51" si="5">$H$62/D47</f>
-        <v>3.4836027503452773</v>
+        <v>3.4833901687058213</v>
       </c>
       <c r="M47" s="464">
         <f t="shared" si="5"/>
-        <v>3.3145784603028727</v>
+        <v>3.3143100573862188</v>
       </c>
       <c r="N47" s="464">
         <f t="shared" si="5"/>
-        <v>3.1611972733248908</v>
+        <v>3.1608840551227209</v>
       </c>
       <c r="O47" s="464">
         <f t="shared" si="5"/>
-        <v>3.0213835963017721</v>
+        <v>3.0210343676453819</v>
       </c>
       <c r="P47" s="465">
         <f t="shared" si="5"/>
-        <v>2.8934134814944437</v>
+        <v>2.8930353392109631</v>
       </c>
     </row>
     <row r="48" spans="1:16" ht="16.5" customHeight="1">
-      <c r="B48" s="505"/>
+      <c r="B48" s="506"/>
       <c r="C48" s="199">
         <f>C37</f>
         <v>0.1</v>
       </c>
       <c r="D48" s="457">
         <f t="shared" si="4"/>
-        <v>611.9578424058958</v>
+        <v>612.01533490079305</v>
       </c>
       <c r="E48" s="458">
         <f t="shared" si="4"/>
-        <v>642.86170035609064</v>
+        <v>642.93533653054635</v>
       </c>
       <c r="F48" s="458">
         <f t="shared" si="4"/>
-        <v>673.76555830628524</v>
+        <v>673.85533816029942</v>
       </c>
       <c r="G48" s="458">
         <f t="shared" si="4"/>
-        <v>704.66941625647974</v>
+        <v>704.77533979005227</v>
       </c>
       <c r="H48" s="459">
         <f t="shared" si="4"/>
-        <v>735.57327420667445</v>
-      </c>
-      <c r="J48" s="506"/>
+        <v>735.69534141980546</v>
+      </c>
+      <c r="J48" s="507"/>
       <c r="K48" s="199">
         <f>K37</f>
         <v>0.1</v>
       </c>
       <c r="L48" s="466">
         <f t="shared" si="5"/>
-        <v>3.5950188845538102</v>
+        <v>3.5946811698053569</v>
       </c>
       <c r="M48" s="467">
         <f t="shared" si="5"/>
-        <v>3.4221979607455029</v>
+        <v>3.421806012206138</v>
       </c>
       <c r="N48" s="467">
         <f t="shared" si="5"/>
-        <v>3.2652307213956875</v>
+        <v>3.264795684495498</v>
       </c>
       <c r="O48" s="467">
         <f t="shared" si="5"/>
-        <v>3.122031337314719</v>
+        <v>3.1215621146099761</v>
       </c>
       <c r="P48" s="468">
         <f t="shared" si="5"/>
-        <v>2.9908645095524022</v>
+        <v>2.990368262702682</v>
       </c>
     </row>
     <row r="49" spans="2:17" ht="16.5" customHeight="1">
-      <c r="B49" s="505"/>
+      <c r="B49" s="506"/>
       <c r="C49" s="209">
         <f>C38</f>
         <v>0.11</v>
       </c>
       <c r="D49" s="457">
         <f t="shared" si="4"/>
-        <v>593.29056108458656</v>
+        <v>593.36531842234331</v>
       </c>
       <c r="E49" s="458">
         <f t="shared" si="4"/>
-        <v>622.95748637493227</v>
+        <v>623.04921317110006</v>
       </c>
       <c r="F49" s="474">
         <f t="shared" si="4"/>
-        <v>652.62441166527788</v>
+        <v>652.73310791985659</v>
       </c>
       <c r="G49" s="458">
         <f t="shared" si="4"/>
-        <v>682.29133695562348</v>
+        <v>682.41700266861324</v>
       </c>
       <c r="H49" s="459">
         <f t="shared" si="4"/>
-        <v>711.95826224596919</v>
-      </c>
-      <c r="J49" s="506"/>
+        <v>712.10089741736988</v>
+      </c>
+      <c r="J49" s="507"/>
       <c r="K49" s="209">
         <f>K38</f>
         <v>0.11</v>
       </c>
       <c r="L49" s="466">
         <f t="shared" si="5"/>
-        <v>3.7081324806149105</v>
+        <v>3.7076652977451108</v>
       </c>
       <c r="M49" s="467">
         <f t="shared" si="5"/>
-        <v>3.5315411534775443</v>
+        <v>3.5310212315376797</v>
       </c>
       <c r="N49" s="475">
         <f t="shared" si="5"/>
-        <v>3.3710047627338064</v>
+        <v>3.3704434068175364</v>
       </c>
       <c r="O49" s="467">
         <f t="shared" si="5"/>
-        <v>3.2244290390910959</v>
+        <v>3.2238352669948589</v>
       </c>
       <c r="P49" s="468">
         <f t="shared" si="5"/>
-        <v>3.0900687816443071</v>
+        <v>3.0894498349586499</v>
       </c>
     </row>
     <row r="50" spans="2:17" ht="16.5" customHeight="1">
-      <c r="B50" s="505"/>
+      <c r="B50" s="506"/>
       <c r="C50" s="199">
         <f>C39</f>
         <v>0.12</v>
       </c>
       <c r="D50" s="457">
         <f t="shared" si="4"/>
-        <v>575.47798017649052</v>
+        <v>575.56844818824322</v>
       </c>
       <c r="E50" s="458">
         <f t="shared" si="4"/>
-        <v>603.96791683625327</v>
+        <v>604.0760819973741</v>
       </c>
       <c r="F50" s="458">
         <f t="shared" si="4"/>
-        <v>632.45785349601613</v>
+        <v>632.5837158065051</v>
       </c>
       <c r="G50" s="458">
         <f t="shared" si="4"/>
-        <v>660.94779015577888</v>
+        <v>661.09134961563609</v>
       </c>
       <c r="H50" s="459">
         <f t="shared" si="4"/>
-        <v>689.43772681554174</v>
-      </c>
-      <c r="J50" s="506"/>
+        <v>689.59898342476697</v>
+      </c>
+      <c r="J50" s="507"/>
       <c r="K50" s="199">
         <f>K39</f>
         <v>0.12</v>
       </c>
       <c r="L50" s="466">
         <f t="shared" si="5"/>
-        <v>3.8229090873734086</v>
+        <v>3.8223082014399727</v>
       </c>
       <c r="M50" s="467">
         <f t="shared" si="5"/>
-        <v>3.642577591743934</v>
+        <v>3.641925356034148</v>
       </c>
       <c r="N50" s="467">
         <f t="shared" si="5"/>
-        <v>3.4784926581892113</v>
+        <v>3.4778005582947014</v>
       </c>
       <c r="O50" s="467">
         <f t="shared" si="5"/>
-        <v>3.3285533785981518</v>
+        <v>3.3278305657442018</v>
       </c>
       <c r="P50" s="468">
         <f t="shared" si="5"/>
-        <v>3.1910061118378681</v>
+        <v>3.190259923345744</v>
       </c>
     </row>
     <row r="51" spans="2:17" ht="16.5" customHeight="1">
-      <c r="B51" s="505"/>
+      <c r="B51" s="506"/>
       <c r="C51" s="199">
         <f>C40</f>
         <v>0.13</v>
       </c>
       <c r="D51" s="460">
         <f t="shared" si="4"/>
-        <v>558.47305123726005</v>
+        <v>558.57779796883267</v>
       </c>
       <c r="E51" s="461">
         <f t="shared" si="4"/>
-        <v>585.84254140540747</v>
+        <v>585.96562323072271</v>
       </c>
       <c r="F51" s="461">
         <f t="shared" si="4"/>
-        <v>613.21203157355467</v>
+        <v>613.35344849261276</v>
       </c>
       <c r="G51" s="461">
         <f t="shared" si="4"/>
-        <v>640.58152174170198</v>
+        <v>640.7412737545028</v>
       </c>
       <c r="H51" s="462">
         <f t="shared" si="4"/>
-        <v>667.9510119098494</v>
-      </c>
-      <c r="J51" s="506"/>
+        <v>668.12909901639284</v>
+      </c>
+      <c r="J51" s="507"/>
       <c r="K51" s="199">
         <f>K40</f>
         <v>0.13</v>
       </c>
       <c r="L51" s="469">
         <f t="shared" si="5"/>
-        <v>3.9393127298193633</v>
+        <v>3.9385740142195105</v>
       </c>
       <c r="M51" s="470">
         <f t="shared" si="5"/>
-        <v>3.7552752565942176</v>
+        <v>3.7544864626533809</v>
       </c>
       <c r="N51" s="470">
         <f t="shared" si="5"/>
-        <v>3.5876660709911565</v>
+        <v>3.5868388861377647</v>
       </c>
       <c r="O51" s="470">
         <f t="shared" si="5"/>
-        <v>3.4343794276462027</v>
+        <v>3.4335231553117027</v>
       </c>
       <c r="P51" s="471">
         <f t="shared" si="5"/>
-        <v>3.2936547153504798</v>
+        <v>3.2927768050198662</v>
       </c>
     </row>
     <row r="52" spans="2:17" ht="16.5">
@@ -24123,8 +24117,8 @@
     <mergeCell ref="J36:J40"/>
     <mergeCell ref="B47:B51"/>
   </mergeCells>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.40157480314960631" right="0.40157480314960631" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="92" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -24317,7 +24311,7 @@
       <c r="D16" s="13"/>
     </row>
   </sheetData>
-  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.31496062992125984" bottom="0.27559055118110237" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.40157480314960631" right="0.47244094488188981" top="0.40157480314960631" bottom="0.40157480314960631" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>